<commit_message>
Feat: Re-generate 100% full text English EDA reports with complete tables and appendices
</commit_message>
<xml_diff>
--- a/BIZ-Jeonbok/data/BIZ_Abalone_Integrated_Data_EN.xlsx
+++ b/BIZ-Jeonbok/data/BIZ_Abalone_Integrated_Data_EN.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Abalone_Trade_Summary_EN" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Size_Pricing_Matrix_EN" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,13 +31,25 @@
       <color rgb="001F497D"/>
       <sz val="15"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F497D"/>
+        <bgColor rgb="001F497D"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -52,9 +64,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -420,13 +433,205 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>📊 Korean Abalone Global Trade EDA Dashboard (English Version)</t>
+          <t>📊 Korean Abalone Size Specification &amp; Global Price Structure Matrix (English)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Grade / Size Spec</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Piece Weight</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Major Exporters</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Avg CIF Price ($/kg)</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Target Market &amp; Buyer Channel</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Sourcing Strategy</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Under 10 pcs/kg (Large)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>100g+ / pc</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Korea, Australia</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>$42.0 ~ $48.0</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Japan High-end Omakase, Ryokan</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Premium Air Direct Express Offer</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>10 ~ 12 pcs/kg (Med-Large)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>80g ~ 100g</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Korea (Wando)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>$36.0 ~ $40.0</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Tokyo Toyosu Wholesalers, LA</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Primary Export Grade, 1st Tier Wholesalers</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>13 ~ 15 pcs/kg (Medium)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>65g ~ 80g</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Korea, China</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>$30.0 ~ $34.0</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Kansai Restaurants, Asian Marts</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>H-Mart, 99 Ranch Supermarket Supply</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>15 ~ 20 pcs/kg (Med-Small)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>50g ~ 65g</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Korea, Vietnam</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>$24.0 ~ $28.0</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Frozen IQF Processors, Foodservice</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Sea Reefer Container FCL Bulk Supply</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>20+ pcs/kg (Small/Process)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Under 50g</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Korea, China</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>$18.0 ~ $22.0</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Canned Abalone, HMR Retort</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>FDA LACF Certified Processing Plants</t>
         </is>
       </c>
     </row>

</xml_diff>